<commit_message>
Updates from UTA and LSC
</commit_message>
<xml_diff>
--- a/AuthorList.xlsx
+++ b/AuthorList.xlsx
@@ -3266,7 +3266,9 @@
       <c r="F66" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="G66" s="2"/>
+      <c r="G66" s="7" t="n">
+        <v>46366</v>
+      </c>
       <c r="H66" s="3" t="s">
         <v>131</v>
       </c>
@@ -3663,7 +3665,9 @@
       <c r="F84" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="G84" s="2"/>
+      <c r="G84" s="7" t="n">
+        <v>46031</v>
+      </c>
       <c r="H84" s="3" t="s">
         <v>318</v>
       </c>

</xml_diff>

<commit_message>
Last active day for HU members
</commit_message>
<xml_diff>
--- a/AuthorList.xlsx
+++ b/AuthorList.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -1551,37 +1551,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546a"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e7e6e6"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472c4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ed7d31"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="ffc000"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5b9bd5"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70ad47"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563c1"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954f72"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -1721,7 +1721,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K1048576"/>
-  <sheetFormatPr defaultColWidth="10.55078125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.55078125" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="20.83"/>
@@ -2653,7 +2653,9 @@
       <c r="F41" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="G41" s="4"/>
+      <c r="G41" s="7" t="n">
+        <v>46258</v>
+      </c>
       <c r="H41" s="5" t="s">
         <v>202</v>
       </c>
@@ -3657,7 +3659,9 @@
       <c r="F87" s="3" t="s">
         <v>368</v>
       </c>
-      <c r="G87" s="4"/>
+      <c r="G87" s="7" t="n">
+        <v>46258</v>
+      </c>
       <c r="H87" s="5" t="s">
         <v>202</v>
       </c>

</xml_diff>

<commit_message>
Updates in EHU and legacy of R. Felkai extended
</commit_message>
<xml_diff>
--- a/AuthorList.xlsx
+++ b/AuthorList.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="440">
   <si>
     <t xml:space="preserve">LastName</t>
   </si>
@@ -401,6 +401,15 @@
   </si>
   <si>
     <t xml:space="preserve">Manchester. M13 9PL, United Kingdom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cruz-Gutiérrez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">angel.cruz@ehu.eus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://orcid.org/0009-0003-7906-0160</t>
   </si>
   <si>
     <t xml:space="preserve">Dey</t>
@@ -1341,7 +1350,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1366,6 +1375,13 @@
     </font>
     <font>
       <u val="single"/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="10"/>
       <name val="Calibri"/>
@@ -1433,7 +1449,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1466,7 +1482,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1867,7 +1891,9 @@
       <c r="F6" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="G6" s="4"/>
+      <c r="G6" s="7" t="n">
+        <v>46307</v>
+      </c>
       <c r="H6" s="5" t="s">
         <v>39</v>
       </c>
@@ -1888,7 +1914,7 @@
       <c r="F7" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="8" t="s">
         <v>44</v>
       </c>
       <c r="H7" s="5" t="s">
@@ -1974,7 +2000,7 @@
       <c r="F11" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="8" t="s">
         <v>67</v>
       </c>
       <c r="H11" s="5" t="s">
@@ -2065,7 +2091,7 @@
       <c r="F15" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="G15" s="7" t="s">
+      <c r="G15" s="8" t="s">
         <v>88</v>
       </c>
       <c r="H15" s="5" t="s">
@@ -2285,58 +2311,58 @@
         <v>127</v>
       </c>
       <c r="B25" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E25" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="F25" s="9" t="s">
         <v>129</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>130</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="5" t="s">
-        <v>131</v>
+        <v>39</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>132</v>
+        <v>16</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="F26" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="G26" s="4"/>
+      <c r="H26" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="I26" s="5" t="s">
         <v>135</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="G26" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="H26" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I26" s="5" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E27" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="E27" s="3" t="s">
+      <c r="F27" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="F27" s="3"/>
-      <c r="G27" s="7" t="n">
-        <v>46240</v>
+      <c r="G27" s="6" t="s">
+        <v>140</v>
       </c>
       <c r="H27" s="5" t="s">
         <v>15</v>
@@ -2347,16 +2373,17 @@
     </row>
     <row r="28" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="F28" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E28" s="3" t="s">
         <v>142</v>
+      </c>
+      <c r="F28" s="3"/>
+      <c r="G28" s="8" t="n">
+        <v>46240</v>
       </c>
       <c r="H28" s="5" t="s">
         <v>15</v>
@@ -2364,99 +2391,98 @@
       <c r="I28" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="J28" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="K28" s="5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="29" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
         <v>143</v>
       </c>
       <c r="B29" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="F29" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="F29" s="1" t="s">
+      <c r="H29" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="J29" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="K29" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="H29" s="1" t="s">
+      <c r="B30" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="H30" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="I29" s="1" t="s">
+      <c r="I30" s="1" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="G30" s="6" t="n">
-        <v>45779</v>
-      </c>
-      <c r="H30" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I30" s="5" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E31" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="F31" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="G31" s="6" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I31" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="F31" s="3" t="s">
+    </row>
+    <row r="32" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="G31" s="4"/>
-      <c r="H31" s="5" t="s">
+      <c r="B32" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="I31" s="5" t="s">
+      <c r="E32" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="G32" s="4"/>
+      <c r="H32" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="I32" s="5" t="s">
         <v>113</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="F32" s="3"/>
-      <c r="G32" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="H32" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I32" s="5" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2464,125 +2490,123 @@
         <v>160</v>
       </c>
       <c r="B33" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="F33" s="3"/>
+      <c r="G33" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="F33" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="H33" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="I33" s="1" t="s">
-        <v>132</v>
+      <c r="H33" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="E34" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="F34" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="H34" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="F34" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="H34" s="1" t="s">
-        <v>169</v>
-      </c>
       <c r="I34" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="J34" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="K34" s="1" t="s">
-        <v>171</v>
+        <v>135</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="H35" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="I35" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="J35" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="K35" s="1" t="s">
         <v>174</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="I35" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="E36" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="F36" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="H36" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="B37" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="H36" s="1" t="s">
+      <c r="C37" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="H37" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I36" s="1" t="s">
+      <c r="I37" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J36" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="K36" s="1" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="F37" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="G37" s="7" t="n">
-        <v>46307</v>
-      </c>
-      <c r="H37" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="I37" s="5" t="s">
-        <v>126</v>
+      <c r="J37" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="K37" s="1" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>144</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>186</v>
@@ -2590,7 +2614,9 @@
       <c r="F38" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="G38" s="4"/>
+      <c r="G38" s="8" t="n">
+        <v>46307</v>
+      </c>
       <c r="H38" s="5" t="s">
         <v>125</v>
       </c>
@@ -2603,129 +2629,129 @@
         <v>188</v>
       </c>
       <c r="B39" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="E39" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="E39" s="3" t="s">
+      <c r="F39" s="3" t="s">
         <v>190</v>
-      </c>
-      <c r="F39" s="3" t="s">
-        <v>191</v>
       </c>
       <c r="G39" s="4"/>
       <c r="H39" s="5" t="s">
-        <v>192</v>
+        <v>125</v>
       </c>
       <c r="I39" s="5" t="s">
-        <v>193</v>
+        <v>126</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="F40" s="3" t="s">
         <v>194</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>197</v>
       </c>
       <c r="G40" s="4"/>
       <c r="H40" s="5" t="s">
-        <v>51</v>
+        <v>195</v>
       </c>
       <c r="I40" s="5" t="s">
-        <v>52</v>
+        <v>196</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="E41" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="E41" s="3" t="s">
+      <c r="F41" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="F41" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="G41" s="7" t="n">
-        <v>46258</v>
-      </c>
+      <c r="G41" s="4"/>
       <c r="H41" s="5" t="s">
-        <v>202</v>
+        <v>51</v>
       </c>
       <c r="I41" s="5" t="s">
-        <v>203</v>
+        <v>52</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="F42" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="G42" s="8" t="n">
+        <v>46258</v>
+      </c>
+      <c r="H42" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="E42" s="3" t="s">
+      <c r="I42" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="F42" s="3" t="s">
+    </row>
+    <row r="43" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="G42" s="4"/>
-      <c r="H42" s="5" t="s">
+      <c r="B43" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="G43" s="4"/>
+      <c r="H43" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="I42" s="5" t="s">
+      <c r="I43" s="5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="G43" s="2" t="n">
-        <v>46307</v>
-      </c>
-      <c r="H43" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="I43" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
         <v>211</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E44" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E44" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="F44" s="3" t="s">
+      <c r="F44" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="G44" s="4"/>
-      <c r="H44" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I44" s="5" t="s">
-        <v>151</v>
+      <c r="G44" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="H44" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2733,46 +2759,44 @@
         <v>214</v>
       </c>
       <c r="B45" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E45" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="E45" s="3" t="s">
+      <c r="F45" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="F45" s="5" t="s">
-        <v>217</v>
-      </c>
+      <c r="G45" s="4"/>
       <c r="H45" s="5" t="s">
-        <v>125</v>
+        <v>27</v>
       </c>
       <c r="I45" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="J45" s="5"/>
-      <c r="K45" s="5" t="s">
-        <v>126</v>
+        <v>154</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="B46" s="1" t="s">
         <v>218</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="E46" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="F46" s="3" t="s">
+      <c r="F46" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="G46" s="7" t="n">
-        <v>46307</v>
-      </c>
       <c r="H46" s="5" t="s">
-        <v>45</v>
+        <v>125</v>
       </c>
       <c r="I46" s="5" t="s">
-        <v>46</v>
+        <v>126</v>
+      </c>
+      <c r="J46" s="5"/>
+      <c r="K46" s="5" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2780,40 +2804,42 @@
         <v>221</v>
       </c>
       <c r="B47" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E47" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="E47" s="3" t="s">
+      <c r="F47" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="F47" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="G47" s="7" t="s">
-        <v>225</v>
+      <c r="G47" s="8" t="n">
+        <v>46307</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="I47" s="5" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="E48" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="B48" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="E48" s="3" t="s">
+      <c r="F48" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="F48" s="3" t="s">
+      <c r="G48" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="G48" s="4"/>
       <c r="H48" s="5" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="I48" s="5" t="s">
         <v>16</v>
@@ -2824,7 +2850,7 @@
         <v>229</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>199</v>
+        <v>85</v>
       </c>
       <c r="E49" s="3" t="s">
         <v>230</v>
@@ -2832,33 +2858,35 @@
       <c r="F49" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="G49" s="4"/>
+      <c r="G49" s="7" t="n">
+        <v>46307</v>
+      </c>
       <c r="H49" s="5" t="s">
-        <v>232</v>
+        <v>39</v>
       </c>
       <c r="I49" s="5" t="s">
-        <v>233</v>
+        <v>16</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="F50" s="3" t="s">
         <v>234</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E50" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="F50" s="3" t="s">
-        <v>236</v>
       </c>
       <c r="G50" s="4"/>
       <c r="H50" s="5" t="s">
-        <v>15</v>
+        <v>235</v>
       </c>
       <c r="I50" s="5" t="s">
-        <v>16</v>
+        <v>236</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2866,28 +2894,28 @@
         <v>237</v>
       </c>
       <c r="B51" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E51" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="E51" s="3" t="s">
+      <c r="F51" s="3" t="s">
         <v>239</v>
-      </c>
-      <c r="F51" s="3" t="s">
-        <v>240</v>
       </c>
       <c r="G51" s="4"/>
       <c r="H51" s="5" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="I51" s="5" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="B52" s="1" t="s">
         <v>241</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>122</v>
       </c>
       <c r="E52" s="3" t="s">
         <v>242</v>
@@ -2897,10 +2925,10 @@
       </c>
       <c r="G52" s="4"/>
       <c r="H52" s="5" t="s">
-        <v>164</v>
+        <v>45</v>
       </c>
       <c r="I52" s="5" t="s">
-        <v>132</v>
+        <v>46</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2908,7 +2936,7 @@
         <v>244</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>85</v>
+        <v>122</v>
       </c>
       <c r="E53" s="3" t="s">
         <v>245</v>
@@ -2918,10 +2946,10 @@
       </c>
       <c r="G53" s="4"/>
       <c r="H53" s="5" t="s">
-        <v>39</v>
+        <v>167</v>
       </c>
       <c r="I53" s="5" t="s">
-        <v>16</v>
+        <v>135</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2929,62 +2957,64 @@
         <v>247</v>
       </c>
       <c r="B54" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E54" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="E54" s="3" t="s">
+      <c r="F54" s="3" t="s">
         <v>249</v>
       </c>
-      <c r="F54" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="G54" s="4"/>
+      <c r="G54" s="7" t="n">
+        <v>46307</v>
+      </c>
       <c r="H54" s="5" t="s">
-        <v>82</v>
+        <v>39</v>
       </c>
       <c r="I54" s="5" t="s">
-        <v>113</v>
+        <v>16</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B55" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="E55" s="3" t="s">
         <v>252</v>
       </c>
-      <c r="E55" s="3" t="s">
+      <c r="F55" s="3" t="s">
         <v>253</v>
-      </c>
-      <c r="F55" s="3" t="s">
-        <v>254</v>
       </c>
       <c r="G55" s="4"/>
       <c r="H55" s="5" t="s">
-        <v>45</v>
+        <v>82</v>
       </c>
       <c r="I55" s="5" t="s">
-        <v>255</v>
+        <v>113</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="E56" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="B56" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="E56" s="3" t="s">
+      <c r="F56" s="3" t="s">
         <v>257</v>
-      </c>
-      <c r="F56" s="3" t="s">
-        <v>258</v>
       </c>
       <c r="G56" s="4"/>
       <c r="H56" s="5" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="I56" s="5" t="s">
-        <v>22</v>
+        <v>258</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2992,91 +3022,91 @@
         <v>259</v>
       </c>
       <c r="B57" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E57" s="3" t="s">
         <v>260</v>
       </c>
-      <c r="E57" s="3" t="s">
+      <c r="F57" s="3" t="s">
         <v>261</v>
-      </c>
-      <c r="F57" s="3" t="s">
-        <v>262</v>
       </c>
       <c r="G57" s="4"/>
       <c r="H57" s="5" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="I57" s="5" t="s">
-        <v>255</v>
+        <v>22</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="B58" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="E58" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="E58" s="3" t="s">
+      <c r="F58" s="3" t="s">
         <v>265</v>
-      </c>
-      <c r="F58" s="3" t="s">
-        <v>266</v>
       </c>
       <c r="G58" s="4"/>
       <c r="H58" s="5" t="s">
         <v>45</v>
       </c>
       <c r="I58" s="5" t="s">
-        <v>46</v>
+        <v>258</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="B59" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="E59" s="3" t="s">
         <v>268</v>
       </c>
-      <c r="E59" s="3" t="s">
+      <c r="F59" s="3" t="s">
         <v>269</v>
-      </c>
-      <c r="F59" s="3" t="s">
-        <v>270</v>
       </c>
       <c r="G59" s="4"/>
       <c r="H59" s="5" t="s">
-        <v>164</v>
+        <v>45</v>
       </c>
       <c r="I59" s="5" t="s">
-        <v>132</v>
+        <v>46</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="B60" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="E60" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="E60" s="3" t="s">
+      <c r="F60" s="3" t="s">
         <v>273</v>
-      </c>
-      <c r="F60" s="3" t="s">
-        <v>274</v>
       </c>
       <c r="G60" s="4"/>
       <c r="H60" s="5" t="s">
-        <v>131</v>
+        <v>167</v>
       </c>
       <c r="I60" s="5" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="B61" s="1" t="s">
         <v>275</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>173</v>
       </c>
       <c r="E61" s="3" t="s">
         <v>276</v>
@@ -3086,10 +3116,10 @@
       </c>
       <c r="G61" s="4"/>
       <c r="H61" s="5" t="s">
-        <v>39</v>
+        <v>134</v>
       </c>
       <c r="I61" s="5" t="s">
-        <v>16</v>
+        <v>135</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3097,141 +3127,143 @@
         <v>278</v>
       </c>
       <c r="B62" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="E62" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="E62" s="3" t="s">
+      <c r="F62" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="F62" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="G62" s="4"/>
+      <c r="G62" s="7" t="n">
+        <v>46307</v>
+      </c>
       <c r="H62" s="5" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="I62" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="J62" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="K62" s="5" t="s">
-        <v>171</v>
-      </c>
     </row>
     <row r="63" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="B63" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="E63" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="E63" s="3" t="s">
+      <c r="F63" s="3" t="s">
         <v>284</v>
-      </c>
-      <c r="F63" s="3" t="s">
-        <v>285</v>
       </c>
       <c r="G63" s="4"/>
       <c r="H63" s="5" t="s">
-        <v>156</v>
+        <v>15</v>
       </c>
       <c r="I63" s="5" t="s">
-        <v>113</v>
+        <v>16</v>
+      </c>
+      <c r="J63" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="K63" s="5" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="B64" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="B64" s="1" t="s">
+      <c r="E64" s="3" t="s">
         <v>287</v>
       </c>
-      <c r="E64" s="3" t="s">
+      <c r="F64" s="3" t="s">
         <v>288</v>
-      </c>
-      <c r="F64" s="3" t="s">
-        <v>289</v>
       </c>
       <c r="G64" s="4"/>
       <c r="H64" s="5" t="s">
-        <v>21</v>
+        <v>159</v>
       </c>
       <c r="I64" s="5" t="s">
-        <v>22</v>
+        <v>113</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="B65" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="B65" s="1" t="s">
+      <c r="E65" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="E65" s="3" t="s">
+      <c r="F65" s="3" t="s">
         <v>292</v>
       </c>
-      <c r="F65" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="G65" s="7" t="n">
-        <v>46307</v>
-      </c>
+      <c r="G65" s="4"/>
       <c r="H65" s="5" t="s">
-        <v>131</v>
+        <v>21</v>
       </c>
       <c r="I65" s="5" t="s">
-        <v>132</v>
+        <v>22</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="B66" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="B66" s="1" t="s">
+      <c r="E66" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="E66" s="3" t="s">
+      <c r="F66" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="F66" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="G66" s="4"/>
+      <c r="G66" s="8" t="n">
+        <v>46307</v>
+      </c>
       <c r="H66" s="5" t="s">
-        <v>45</v>
+        <v>134</v>
       </c>
       <c r="I66" s="5" t="s">
-        <v>46</v>
+        <v>135</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="B67" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="B67" s="1" t="s">
+      <c r="E67" s="3" t="s">
         <v>299</v>
       </c>
-      <c r="E67" s="3" t="s">
+      <c r="F67" s="3" t="s">
         <v>300</v>
-      </c>
-      <c r="F67" s="3" t="s">
-        <v>301</v>
       </c>
       <c r="G67" s="4"/>
       <c r="H67" s="5" t="s">
-        <v>131</v>
+        <v>45</v>
       </c>
       <c r="I67" s="5" t="s">
-        <v>132</v>
+        <v>46</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="B68" s="1" t="s">
         <v>302</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>128</v>
       </c>
       <c r="E68" s="3" t="s">
         <v>303</v>
@@ -3241,10 +3273,10 @@
       </c>
       <c r="G68" s="4"/>
       <c r="H68" s="5" t="s">
-        <v>15</v>
+        <v>134</v>
       </c>
       <c r="I68" s="5" t="s">
-        <v>16</v>
+        <v>135</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3252,28 +3284,28 @@
         <v>305</v>
       </c>
       <c r="B69" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="E69" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="E69" s="3" t="s">
+      <c r="F69" s="3" t="s">
         <v>307</v>
-      </c>
-      <c r="F69" s="3" t="s">
-        <v>308</v>
       </c>
       <c r="G69" s="4"/>
       <c r="H69" s="5" t="s">
-        <v>125</v>
+        <v>15</v>
       </c>
       <c r="I69" s="5" t="s">
-        <v>126</v>
+        <v>16</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="B70" s="1" t="s">
         <v>309</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>173</v>
       </c>
       <c r="E70" s="3" t="s">
         <v>310</v>
@@ -3283,50 +3315,52 @@
       </c>
       <c r="G70" s="4"/>
       <c r="H70" s="5" t="s">
-        <v>312</v>
+        <v>125</v>
       </c>
       <c r="I70" s="5" t="s">
-        <v>313</v>
+        <v>126</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="F71" s="3" t="s">
         <v>314</v>
-      </c>
-      <c r="B71" s="1" t="s">
-        <v>315</v>
-      </c>
-      <c r="E71" s="3" t="s">
-        <v>316</v>
-      </c>
-      <c r="F71" s="3" t="s">
-        <v>317</v>
       </c>
       <c r="G71" s="4"/>
       <c r="H71" s="5" t="s">
-        <v>125</v>
+        <v>315</v>
       </c>
       <c r="I71" s="5" t="s">
-        <v>126</v>
+        <v>316</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="B72" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="B72" s="1" t="s">
+      <c r="E72" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="E72" s="3" t="s">
+      <c r="F72" s="3" t="s">
         <v>320</v>
       </c>
-      <c r="F72" s="3"/>
       <c r="G72" s="4"/>
       <c r="H72" s="5" t="s">
-        <v>232</v>
+        <v>125</v>
       </c>
       <c r="I72" s="5" t="s">
-        <v>233</v>
+        <v>126</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3334,20 +3368,18 @@
         <v>321</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>85</v>
+        <v>322</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="F73" s="3" t="s">
         <v>323</v>
       </c>
+      <c r="F73" s="3"/>
       <c r="G73" s="4"/>
       <c r="H73" s="5" t="s">
-        <v>169</v>
+        <v>235</v>
       </c>
       <c r="I73" s="5" t="s">
-        <v>16</v>
+        <v>236</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3355,7 +3387,7 @@
         <v>324</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>173</v>
+        <v>85</v>
       </c>
       <c r="E74" s="3" t="s">
         <v>325</v>
@@ -3365,7 +3397,7 @@
       </c>
       <c r="G74" s="4"/>
       <c r="H74" s="5" t="s">
-        <v>15</v>
+        <v>172</v>
       </c>
       <c r="I74" s="5" t="s">
         <v>16</v>
@@ -3376,7 +3408,7 @@
         <v>327</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>69</v>
+        <v>176</v>
       </c>
       <c r="E75" s="3" t="s">
         <v>328</v>
@@ -3386,10 +3418,10 @@
       </c>
       <c r="G75" s="4"/>
       <c r="H75" s="5" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="I75" s="5" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3397,7 +3429,7 @@
         <v>330</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>264</v>
+        <v>69</v>
       </c>
       <c r="E76" s="3" t="s">
         <v>331</v>
@@ -3407,10 +3439,10 @@
       </c>
       <c r="G76" s="4"/>
       <c r="H76" s="5" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="I76" s="5" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3418,7 +3450,7 @@
         <v>333</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>252</v>
+        <v>267</v>
       </c>
       <c r="E77" s="3" t="s">
         <v>334</v>
@@ -3439,7 +3471,7 @@
         <v>336</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>306</v>
+        <v>255</v>
       </c>
       <c r="E78" s="3" t="s">
         <v>337</v>
@@ -3449,16 +3481,10 @@
       </c>
       <c r="G78" s="4"/>
       <c r="H78" s="5" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I78" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J78" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="K78" s="5" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3466,7 +3492,7 @@
         <v>339</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>91</v>
+        <v>309</v>
       </c>
       <c r="E79" s="3" t="s">
         <v>340</v>
@@ -3476,9 +3502,15 @@
       </c>
       <c r="G79" s="4"/>
       <c r="H79" s="5" t="s">
-        <v>89</v>
+        <v>39</v>
       </c>
       <c r="I79" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="J79" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K79" s="5" t="s">
         <v>16</v>
       </c>
     </row>
@@ -3487,24 +3519,20 @@
         <v>342</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>315</v>
-      </c>
-      <c r="C80" s="1"/>
+        <v>91</v>
+      </c>
       <c r="E80" s="3" t="s">
         <v>343</v>
       </c>
       <c r="F80" s="3" t="s">
         <v>344</v>
       </c>
-      <c r="G80" s="6"/>
+      <c r="G80" s="4"/>
       <c r="H80" s="5" t="s">
-        <v>15</v>
+        <v>89</v>
       </c>
       <c r="I80" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="K80" s="5" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3512,33 +3540,35 @@
         <v>345</v>
       </c>
       <c r="B81" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="C81" s="1"/>
+      <c r="E81" s="3" t="s">
         <v>346</v>
       </c>
-      <c r="C81" s="1" t="s">
+      <c r="F81" s="3" t="s">
         <v>347</v>
       </c>
-      <c r="E81" s="3" t="s">
-        <v>348</v>
-      </c>
-      <c r="F81" s="3" t="s">
-        <v>349</v>
-      </c>
-      <c r="G81" s="6" t="n">
-        <v>45779</v>
-      </c>
+      <c r="G81" s="6"/>
       <c r="H81" s="5" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="I81" s="5" t="s">
-        <v>46</v>
+        <v>16</v>
+      </c>
+      <c r="K81" s="5" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="C82" s="1" t="s">
         <v>350</v>
-      </c>
-      <c r="B82" s="1" t="s">
-        <v>128</v>
       </c>
       <c r="E82" s="3" t="s">
         <v>351</v>
@@ -3546,14 +3576,14 @@
       <c r="F82" s="3" t="s">
         <v>352</v>
       </c>
-      <c r="G82" s="7" t="n">
-        <v>46266</v>
+      <c r="G82" s="6" t="n">
+        <v>45779</v>
       </c>
       <c r="H82" s="5" t="s">
-        <v>312</v>
+        <v>45</v>
       </c>
       <c r="I82" s="5" t="s">
-        <v>313</v>
+        <v>46</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3561,7 +3591,7 @@
         <v>353</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E83" s="3" t="s">
         <v>354</v>
@@ -3569,12 +3599,14 @@
       <c r="F83" s="3" t="s">
         <v>355</v>
       </c>
-      <c r="G83" s="4"/>
+      <c r="G83" s="8" t="n">
+        <v>46266</v>
+      </c>
       <c r="H83" s="5" t="s">
-        <v>45</v>
+        <v>315</v>
       </c>
       <c r="I83" s="5" t="s">
-        <v>46</v>
+        <v>316</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3582,25 +3614,25 @@
         <v>356</v>
       </c>
       <c r="B84" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E84" s="3" t="s">
         <v>357</v>
       </c>
-      <c r="E84" s="3" t="s">
+      <c r="F84" s="3" t="s">
         <v>358</v>
-      </c>
-      <c r="F84" s="3" t="s">
-        <v>359</v>
       </c>
       <c r="G84" s="4"/>
       <c r="H84" s="5" t="s">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="I84" s="5" t="s">
-        <v>113</v>
+        <v>46</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="1" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="B85" s="1" t="s">
         <v>360</v>
@@ -3613,7 +3645,7 @@
       </c>
       <c r="G85" s="4"/>
       <c r="H85" s="5" t="s">
-        <v>156</v>
+        <v>82</v>
       </c>
       <c r="I85" s="5" t="s">
         <v>113</v>
@@ -3621,10 +3653,10 @@
     </row>
     <row r="86" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="B86" s="1" t="s">
         <v>363</v>
-      </c>
-      <c r="B86" s="1" t="s">
-        <v>69</v>
       </c>
       <c r="E86" s="3" t="s">
         <v>364</v>
@@ -3634,16 +3666,10 @@
       </c>
       <c r="G86" s="4"/>
       <c r="H86" s="5" t="s">
-        <v>15</v>
+        <v>159</v>
       </c>
       <c r="I86" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J86" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="K86" s="5" t="s">
-        <v>73</v>
+        <v>113</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3651,7 +3677,7 @@
         <v>366</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>306</v>
+        <v>69</v>
       </c>
       <c r="E87" s="3" t="s">
         <v>367</v>
@@ -3659,14 +3685,18 @@
       <c r="F87" s="3" t="s">
         <v>368</v>
       </c>
-      <c r="G87" s="7" t="n">
-        <v>46258</v>
-      </c>
+      <c r="G87" s="4"/>
       <c r="H87" s="5" t="s">
-        <v>202</v>
+        <v>15</v>
       </c>
       <c r="I87" s="5" t="s">
-        <v>203</v>
+        <v>16</v>
+      </c>
+      <c r="J87" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="K87" s="5" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3674,28 +3704,30 @@
         <v>369</v>
       </c>
       <c r="B88" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="E88" s="3" t="s">
         <v>370</v>
       </c>
-      <c r="E88" s="3" t="s">
+      <c r="F88" s="3" t="s">
         <v>371</v>
       </c>
-      <c r="F88" s="3" t="s">
-        <v>372</v>
-      </c>
-      <c r="G88" s="4"/>
+      <c r="G88" s="8" t="n">
+        <v>46258</v>
+      </c>
       <c r="H88" s="5" t="s">
-        <v>57</v>
+        <v>205</v>
       </c>
       <c r="I88" s="5" t="s">
-        <v>58</v>
+        <v>206</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="B89" s="1" t="s">
         <v>373</v>
-      </c>
-      <c r="B89" s="1" t="s">
-        <v>95</v>
       </c>
       <c r="E89" s="3" t="s">
         <v>374</v>
@@ -3705,10 +3737,10 @@
       </c>
       <c r="G89" s="4"/>
       <c r="H89" s="5" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="I89" s="5" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3716,34 +3748,28 @@
         <v>376</v>
       </c>
       <c r="B90" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E90" s="3" t="s">
         <v>377</v>
       </c>
-      <c r="E90" s="3" t="s">
+      <c r="F90" s="3" t="s">
         <v>378</v>
-      </c>
-      <c r="F90" s="3" t="s">
-        <v>379</v>
       </c>
       <c r="G90" s="4"/>
       <c r="H90" s="5" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="I90" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J90" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="K90" s="5" t="s">
-        <v>171</v>
+        <v>46</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="B91" s="1" t="s">
         <v>380</v>
-      </c>
-      <c r="B91" s="1" t="s">
-        <v>264</v>
       </c>
       <c r="E91" s="3" t="s">
         <v>381</v>
@@ -3751,14 +3777,18 @@
       <c r="F91" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="G91" s="7" t="n">
-        <v>46307</v>
-      </c>
+      <c r="G91" s="4"/>
       <c r="H91" s="5" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="I91" s="5" t="s">
-        <v>46</v>
+        <v>16</v>
+      </c>
+      <c r="J91" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="K91" s="5" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3766,7 +3796,7 @@
         <v>383</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>173</v>
+        <v>267</v>
       </c>
       <c r="E92" s="3" t="s">
         <v>384</v>
@@ -3774,7 +3804,9 @@
       <c r="F92" s="3" t="s">
         <v>385</v>
       </c>
-      <c r="G92" s="4"/>
+      <c r="G92" s="8" t="n">
+        <v>46307</v>
+      </c>
       <c r="H92" s="5" t="s">
         <v>45</v>
       </c>
@@ -3787,7 +3819,7 @@
         <v>386</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>41</v>
+        <v>176</v>
       </c>
       <c r="E93" s="3" t="s">
         <v>387</v>
@@ -3808,28 +3840,28 @@
         <v>389</v>
       </c>
       <c r="B94" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E94" s="3" t="s">
         <v>390</v>
       </c>
-      <c r="E94" s="3" t="s">
+      <c r="F94" s="3" t="s">
         <v>391</v>
-      </c>
-      <c r="F94" s="3" t="s">
-        <v>392</v>
       </c>
       <c r="G94" s="4"/>
       <c r="H94" s="5" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="I94" s="5" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="B95" s="1" t="s">
         <v>393</v>
-      </c>
-      <c r="B95" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="E95" s="3" t="s">
         <v>394</v>
@@ -3839,10 +3871,10 @@
       </c>
       <c r="G95" s="4"/>
       <c r="H95" s="5" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="I95" s="5" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3850,7 +3882,7 @@
         <v>396</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>41</v>
+        <v>91</v>
       </c>
       <c r="E96" s="3" t="s">
         <v>397</v>
@@ -3871,7 +3903,7 @@
         <v>399</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>252</v>
+        <v>41</v>
       </c>
       <c r="E97" s="3" t="s">
         <v>400</v>
@@ -3879,91 +3911,87 @@
       <c r="F97" s="3" t="s">
         <v>401</v>
       </c>
-      <c r="G97" s="7" t="s">
-        <v>402</v>
-      </c>
+      <c r="G97" s="4"/>
       <c r="H97" s="5" t="s">
         <v>15</v>
       </c>
       <c r="I97" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="J97" s="5" t="s">
+    </row>
+    <row r="98" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="E98" s="3" t="s">
         <v>403</v>
       </c>
-      <c r="K97" s="5" t="s">
+      <c r="F98" s="3" t="s">
         <v>404</v>
       </c>
-    </row>
-    <row r="98" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="1" t="s">
+      <c r="G98" s="8" t="s">
         <v>405</v>
       </c>
-      <c r="B98" s="1" t="s">
+      <c r="H98" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I98" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="J98" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="K98" s="5" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="B99" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="E98" s="3" t="s">
-        <v>406</v>
-      </c>
-      <c r="F98" s="8" t="s">
-        <v>407</v>
-      </c>
-      <c r="G98" s="7"/>
-      <c r="H98" s="5" t="s">
-        <v>408</v>
-      </c>
-      <c r="I98" s="5" t="s">
+      <c r="E99" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="F99" s="10" t="s">
+        <v>410</v>
+      </c>
+      <c r="G99" s="8"/>
+      <c r="H99" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="I99" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="J98" s="5"/>
-      <c r="K98" s="5"/>
-    </row>
-    <row r="99" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="1" t="s">
-        <v>409</v>
-      </c>
-      <c r="B99" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="E99" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="F99" s="3" t="s">
-        <v>411</v>
-      </c>
-      <c r="G99" s="7" t="n">
-        <v>46307</v>
-      </c>
-      <c r="H99" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="I99" s="5" t="s">
-        <v>126</v>
-      </c>
+      <c r="J99" s="5"/>
+      <c r="K99" s="5"/>
     </row>
     <row r="100" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="1" t="s">
         <v>412</v>
       </c>
       <c r="B100" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E100" s="3" t="s">
         <v>413</v>
       </c>
-      <c r="E100" s="3" t="s">
+      <c r="F100" s="3" t="s">
         <v>414</v>
       </c>
-      <c r="F100" s="3"/>
-      <c r="G100" s="4"/>
+      <c r="G100" s="8" t="n">
+        <v>46307</v>
+      </c>
       <c r="H100" s="5" t="s">
-        <v>15</v>
+        <v>125</v>
       </c>
       <c r="I100" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J100" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="K100" s="5" t="s">
-        <v>16</v>
+        <v>126</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3971,20 +3999,24 @@
         <v>415</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>69</v>
+        <v>416</v>
       </c>
       <c r="E101" s="3" t="s">
-        <v>416</v>
-      </c>
-      <c r="F101" s="3" t="s">
         <v>417</v>
       </c>
+      <c r="F101" s="3"/>
       <c r="G101" s="4"/>
       <c r="H101" s="5" t="s">
-        <v>164</v>
+        <v>15</v>
       </c>
       <c r="I101" s="5" t="s">
-        <v>132</v>
+        <v>16</v>
+      </c>
+      <c r="J101" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="K101" s="5" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3992,7 +4024,7 @@
         <v>418</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>134</v>
+        <v>69</v>
       </c>
       <c r="E102" s="3" t="s">
         <v>419</v>
@@ -4002,16 +4034,10 @@
       </c>
       <c r="G102" s="4"/>
       <c r="H102" s="5" t="s">
-        <v>15</v>
+        <v>167</v>
       </c>
       <c r="I102" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J102" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="K102" s="5" t="s">
-        <v>52</v>
+        <v>135</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4019,70 +4045,76 @@
         <v>421</v>
       </c>
       <c r="B103" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E103" s="3" t="s">
         <v>422</v>
       </c>
-      <c r="E103" s="3" t="s">
+      <c r="F103" s="3" t="s">
         <v>423</v>
-      </c>
-      <c r="F103" s="3" t="s">
-        <v>424</v>
       </c>
       <c r="G103" s="4"/>
       <c r="H103" s="5" t="s">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="I103" s="5" t="s">
-        <v>425</v>
+        <v>16</v>
+      </c>
+      <c r="J103" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="K103" s="5" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="E104" s="3" t="s">
         <v>426</v>
       </c>
-      <c r="B104" s="1" t="s">
+      <c r="F104" s="3" t="s">
         <v>427</v>
-      </c>
-      <c r="E104" s="3" t="s">
-        <v>428</v>
-      </c>
-      <c r="F104" s="3" t="s">
-        <v>429</v>
       </c>
       <c r="G104" s="4"/>
       <c r="H104" s="5" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="I104" s="5" t="s">
-        <v>46</v>
+        <v>428</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="B105" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="B105" s="1" t="s">
+      <c r="E105" s="3" t="s">
         <v>431</v>
       </c>
-      <c r="E105" s="3" t="s">
+      <c r="F105" s="3" t="s">
         <v>432</v>
-      </c>
-      <c r="F105" s="3" t="s">
-        <v>433</v>
       </c>
       <c r="G105" s="4"/>
       <c r="H105" s="5" t="s">
-        <v>125</v>
+        <v>45</v>
       </c>
       <c r="I105" s="5" t="s">
-        <v>126</v>
+        <v>46</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="B106" s="1" t="s">
         <v>434</v>
-      </c>
-      <c r="B106" s="1" t="s">
-        <v>85</v>
       </c>
       <c r="E106" s="3" t="s">
         <v>435</v>
@@ -4092,19 +4124,39 @@
       </c>
       <c r="G106" s="4"/>
       <c r="H106" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I106" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E107" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="F107" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="G107" s="4"/>
+      <c r="H107" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I106" s="5" t="s">
+      <c r="I107" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="J106" s="5" t="s">
+      <c r="J107" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="K106" s="5" t="s">
+      <c r="K107" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
@@ -4134,86 +4186,88 @@
     <hyperlink ref="E22" r:id="rId23" display="Camilo.Cortes@ific.uv.es"/>
     <hyperlink ref="E23" r:id="rId24" display="fp.cossio@ehu.es"/>
     <hyperlink ref="E24" r:id="rId25" display="rhiannon.coupe@postgrad.manchester.ac.uk"/>
-    <hyperlink ref="E25" r:id="rId26" display="exd4668@mavs.uta.edu"/>
-    <hyperlink ref="E26" r:id="rId27" display="pablo.dietz@dipc.org"/>
-    <hyperlink ref="E27" r:id="rId28" display="carlos.echeverria@dipc.org"/>
-    <hyperlink ref="F28" r:id="rId29" display="https://orcid.org/0009-0000-4219-6193"/>
-    <hyperlink ref="E30" r:id="rId30" display="ryan.felkai@gmail.com"/>
-    <hyperlink ref="E31" r:id="rId31" display="pancho@uc.pt"/>
-    <hyperlink ref="E37" r:id="rId32" display="joshua.grocott@postgrad.manchester.ac.uk"/>
-    <hyperlink ref="E38" r:id="rId33" display="roxanne.guenette@manchester.ac.uk"/>
-    <hyperlink ref="E39" r:id="rId34" display="hauptman@iastate.edu"/>
-    <hyperlink ref="E40" r:id="rId35" display="jose.hernando@usc.es"/>
-    <hyperlink ref="E41" r:id="rId36" display="pablo.herrero-gomez@mail.huji.ac.il"/>
-    <hyperlink ref="E42" r:id="rId37" display="viherbos@eln.upv.es"/>
-    <hyperlink ref="E44" r:id="rId38" display="yairifergan@gmail.com"/>
-    <hyperlink ref="E45" r:id="rId39" display="benjamin.jones-7@manchester.ac.uk"/>
-    <hyperlink ref="E46" r:id="rId40" display="fabian.kellerer@ific.uv.es"/>
-    <hyperlink ref="E47" r:id="rId41" display="leire.larizgoitia@dipc.org"/>
-    <hyperlink ref="E48" r:id="rId42" display="amaia.larumbe@ehu.eus"/>
-    <hyperlink ref="E49" r:id="rId43" display="lebrun@fnal.gov"/>
-    <hyperlink ref="E50" r:id="rId44" display="francisco.lopez@dipc.org"/>
-    <hyperlink ref="E51" r:id="rId45" display="lopezneu@ific.uv.es"/>
-    <hyperlink ref="E52" r:id="rId46" display="ryan.madigan@mavs.uta.edu"/>
-    <hyperlink ref="E53" r:id="rId47" display="aimar.marauri@ehu.eus"/>
-    <hyperlink ref="E54" r:id="rId48" display="afonso.marques97@gmail.com"/>
-    <hyperlink ref="E55" r:id="rId49" display="justo.martin-albo@ific.uv.es"/>
-    <hyperlink ref="E56" r:id="rId50" display="alberto.martinez.perez@ific.uv.es"/>
-    <hyperlink ref="E57" r:id="rId51" display="gonzaponte@gmail.com"/>
-    <hyperlink ref="E58" r:id="rId52" display="miryam.martinez@ific.uv.es"/>
-    <hyperlink ref="E59" r:id="rId53" display="rlm6389@mavs.uta.edu"/>
-    <hyperlink ref="E60" r:id="rId54" display="krishan.mistry@uta.edu"/>
-    <hyperlink ref="E61" r:id="rId55" display="juan.molina@ehu.eus"/>
-    <hyperlink ref="E62" r:id="rId56" display="francesc.monrabal@dipc.org"/>
-    <hyperlink ref="E63" r:id="rId57" display="cristinam@uc.pt"/>
-    <hyperlink ref="E64" r:id="rId58" display="fjmora@eln.upv.es"/>
-    <hyperlink ref="E65" r:id="rId59" display="ken6461@mavs.uta.edu"/>
-    <hyperlink ref="F65" r:id="rId60" display="https://orcid.org/0009-0009-0971-5559"/>
-    <hyperlink ref="E66" r:id="rId61" display="pau.novella@ific.uv.es"/>
-    <hyperlink ref="E67" r:id="rId62" display="nygren@uta.edu"/>
-    <hyperlink ref="E68" r:id="rId63" display="eva.oblak@dipc.org"/>
-    <hyperlink ref="E69" r:id="rId64" display="ian.osborne@postgrad.manchester.ac.uk"/>
-    <hyperlink ref="F69" r:id="rId65" display="https://orcid.org/0009-0002-2780-2399"/>
-    <hyperlink ref="E70" r:id="rId66" display="jpalacio@lsc-canfranc.es"/>
-    <hyperlink ref="E71" r:id="rId67" display="brais.palmeiro@manchester.ac.uk"/>
-    <hyperlink ref="E72" r:id="rId68" display="para@fnal.gov"/>
-    <hyperlink ref="E73" r:id="rId69" display="ariadna.pazos@ehu.eus"/>
-    <hyperlink ref="E74" r:id="rId70" display="jorge.pelegrin@dipc.org"/>
-    <hyperlink ref="E75" r:id="rId71" display="martin.maneiro@usc.es"/>
-    <hyperlink ref="E76" r:id="rId72" display="marcque@ific.uv.es"/>
-    <hyperlink ref="E77" r:id="rId73" display="jrenner@ific.uv.es"/>
-    <hyperlink ref="E78" r:id="rId74" display="ivan.rivilla@ehu.es"/>
-    <hyperlink ref="E79" r:id="rId75" display="celia.rogero@csic.es"/>
-    <hyperlink ref="E80" r:id="rId76" display="bromeo@dipc.org"/>
-    <hyperlink ref="E81" r:id="rId77" display="romoluque_c@lanl.gov"/>
-    <hyperlink ref="E82" r:id="rId78" display="eruiz@lsc-canfranc.es"/>
-    <hyperlink ref="E83" r:id="rId79" display="Pokhee.Saharia@ific.uv.es"/>
-    <hyperlink ref="F83" r:id="rId80" display="https://orcid.org/0009-0006-7366-4950"/>
-    <hyperlink ref="E84" r:id="rId81" display="filomena.santos@coimbra.lip.pt"/>
-    <hyperlink ref="E85" r:id="rId82" display="jmf@uc.pt"/>
-    <hyperlink ref="E86" r:id="rId83" display="marc.seemann@dipc.org"/>
-    <hyperlink ref="E87" r:id="rId84" display="itay.shomroni@mail.huji.ac.il"/>
-    <hyperlink ref="E88" r:id="rId85" display="analuisa.silva@ua.pt"/>
-    <hyperlink ref="F88" r:id="rId86" display="https://orcid.org/0000-0002-8363-0109"/>
-    <hyperlink ref="E89" r:id="rId87" display="ander.simon@ific.uv.es"/>
-    <hyperlink ref="E90" r:id="rId88" display="roberto.soleti@dipc.org"/>
-    <hyperlink ref="E91" r:id="rId89" display="sorel@ific.uv.es"/>
-    <hyperlink ref="E92" r:id="rId90" display="josealfonso.soto@ific.uv.es"/>
-    <hyperlink ref="E93" r:id="rId91" display="steruel@ific.uv.es"/>
-    <hyperlink ref="E94" r:id="rId92" display="jtoledo@eln.upv.es"/>
-    <hyperlink ref="E95" r:id="rId93" display="claire.tonnele@dipc.org"/>
-    <hyperlink ref="E96" r:id="rId94" display="samuele.torelli@dipc.org"/>
-    <hyperlink ref="E97" r:id="rId95" display="jordi.torrent@udg.edu"/>
-    <hyperlink ref="F98" r:id="rId96" display="https://orcid.org/0000-0002-7621-5804"/>
-    <hyperlink ref="E99" r:id="rId97" display="alexandra.trettin@manchester.ac.uk"/>
-    <hyperlink ref="E100" r:id="rId98" display="pablo.garcia@dipc.org"/>
-    <hyperlink ref="E101" r:id="rId99" display="mukundam.vanga@uta.edu"/>
-    <hyperlink ref="E102" r:id="rId100" display="pablo.vazquez@dipc.org"/>
-    <hyperlink ref="F102" r:id="rId101" display="https://orcid.org/0009-0007-0098-8927"/>
-    <hyperlink ref="E103" r:id="rId102" display="joao.veloso@ua.pt"/>
-    <hyperlink ref="E104" r:id="rId103" display="Juan.Villamil@ific.uv.es"/>
-    <hyperlink ref="E105" r:id="rId104" display="john.waiton@postgrad.manchester.ac.uk"/>
-    <hyperlink ref="E106" r:id="rId105" display="alfonso.yubero@dipc.org"/>
+    <hyperlink ref="E25" r:id="rId26" display="angel.cruz@ehu.eus"/>
+    <hyperlink ref="F25" r:id="rId27" display="https://orcid.org/0009"/>
+    <hyperlink ref="E26" r:id="rId28" display="exd4668@mavs.uta.edu"/>
+    <hyperlink ref="E27" r:id="rId29" display="pablo.dietz@dipc.org"/>
+    <hyperlink ref="E28" r:id="rId30" display="carlos.echeverria@dipc.org"/>
+    <hyperlink ref="F29" r:id="rId31" display="https://orcid.org/0009-0000-4219-6193"/>
+    <hyperlink ref="E31" r:id="rId32" display="ryan.felkai@gmail.com"/>
+    <hyperlink ref="E32" r:id="rId33" display="pancho@uc.pt"/>
+    <hyperlink ref="E38" r:id="rId34" display="joshua.grocott@postgrad.manchester.ac.uk"/>
+    <hyperlink ref="E39" r:id="rId35" display="roxanne.guenette@manchester.ac.uk"/>
+    <hyperlink ref="E40" r:id="rId36" display="hauptman@iastate.edu"/>
+    <hyperlink ref="E41" r:id="rId37" display="jose.hernando@usc.es"/>
+    <hyperlink ref="E42" r:id="rId38" display="pablo.herrero-gomez@mail.huji.ac.il"/>
+    <hyperlink ref="E43" r:id="rId39" display="viherbos@eln.upv.es"/>
+    <hyperlink ref="E45" r:id="rId40" display="yairifergan@gmail.com"/>
+    <hyperlink ref="E46" r:id="rId41" display="benjamin.jones-7@manchester.ac.uk"/>
+    <hyperlink ref="E47" r:id="rId42" display="fabian.kellerer@ific.uv.es"/>
+    <hyperlink ref="E48" r:id="rId43" display="leire.larizgoitia@dipc.org"/>
+    <hyperlink ref="E49" r:id="rId44" display="amaia.larumbe@ehu.eus"/>
+    <hyperlink ref="E50" r:id="rId45" display="lebrun@fnal.gov"/>
+    <hyperlink ref="E51" r:id="rId46" display="francisco.lopez@dipc.org"/>
+    <hyperlink ref="E52" r:id="rId47" display="lopezneu@ific.uv.es"/>
+    <hyperlink ref="E53" r:id="rId48" display="ryan.madigan@mavs.uta.edu"/>
+    <hyperlink ref="E54" r:id="rId49" display="aimar.marauri@ehu.eus"/>
+    <hyperlink ref="E55" r:id="rId50" display="afonso.marques97@gmail.com"/>
+    <hyperlink ref="E56" r:id="rId51" display="justo.martin-albo@ific.uv.es"/>
+    <hyperlink ref="E57" r:id="rId52" display="alberto.martinez.perez@ific.uv.es"/>
+    <hyperlink ref="E58" r:id="rId53" display="gonzaponte@gmail.com"/>
+    <hyperlink ref="E59" r:id="rId54" display="miryam.martinez@ific.uv.es"/>
+    <hyperlink ref="E60" r:id="rId55" display="rlm6389@mavs.uta.edu"/>
+    <hyperlink ref="E61" r:id="rId56" display="krishan.mistry@uta.edu"/>
+    <hyperlink ref="E62" r:id="rId57" display="juan.molina@ehu.eus"/>
+    <hyperlink ref="E63" r:id="rId58" display="francesc.monrabal@dipc.org"/>
+    <hyperlink ref="E64" r:id="rId59" display="cristinam@uc.pt"/>
+    <hyperlink ref="E65" r:id="rId60" display="fjmora@eln.upv.es"/>
+    <hyperlink ref="E66" r:id="rId61" display="ken6461@mavs.uta.edu"/>
+    <hyperlink ref="F66" r:id="rId62" display="https://orcid.org/0009-0009-0971-5559"/>
+    <hyperlink ref="E67" r:id="rId63" display="pau.novella@ific.uv.es"/>
+    <hyperlink ref="E68" r:id="rId64" display="nygren@uta.edu"/>
+    <hyperlink ref="E69" r:id="rId65" display="eva.oblak@dipc.org"/>
+    <hyperlink ref="E70" r:id="rId66" display="ian.osborne@postgrad.manchester.ac.uk"/>
+    <hyperlink ref="F70" r:id="rId67" display="https://orcid.org/0009-0002-2780-2399"/>
+    <hyperlink ref="E71" r:id="rId68" display="jpalacio@lsc-canfranc.es"/>
+    <hyperlink ref="E72" r:id="rId69" display="brais.palmeiro@manchester.ac.uk"/>
+    <hyperlink ref="E73" r:id="rId70" display="para@fnal.gov"/>
+    <hyperlink ref="E74" r:id="rId71" display="ariadna.pazos@ehu.eus"/>
+    <hyperlink ref="E75" r:id="rId72" display="jorge.pelegrin@dipc.org"/>
+    <hyperlink ref="E76" r:id="rId73" display="martin.maneiro@usc.es"/>
+    <hyperlink ref="E77" r:id="rId74" display="marcque@ific.uv.es"/>
+    <hyperlink ref="E78" r:id="rId75" display="jrenner@ific.uv.es"/>
+    <hyperlink ref="E79" r:id="rId76" display="ivan.rivilla@ehu.es"/>
+    <hyperlink ref="E80" r:id="rId77" display="celia.rogero@csic.es"/>
+    <hyperlink ref="E81" r:id="rId78" display="bromeo@dipc.org"/>
+    <hyperlink ref="E82" r:id="rId79" display="romoluque_c@lanl.gov"/>
+    <hyperlink ref="E83" r:id="rId80" display="eruiz@lsc-canfranc.es"/>
+    <hyperlink ref="E84" r:id="rId81" display="Pokhee.Saharia@ific.uv.es"/>
+    <hyperlink ref="F84" r:id="rId82" display="https://orcid.org/0009-0006-7366-4950"/>
+    <hyperlink ref="E85" r:id="rId83" display="filomena.santos@coimbra.lip.pt"/>
+    <hyperlink ref="E86" r:id="rId84" display="jmf@uc.pt"/>
+    <hyperlink ref="E87" r:id="rId85" display="marc.seemann@dipc.org"/>
+    <hyperlink ref="E88" r:id="rId86" display="itay.shomroni@mail.huji.ac.il"/>
+    <hyperlink ref="E89" r:id="rId87" display="analuisa.silva@ua.pt"/>
+    <hyperlink ref="F89" r:id="rId88" display="https://orcid.org/0000-0002-8363-0109"/>
+    <hyperlink ref="E90" r:id="rId89" display="ander.simon@ific.uv.es"/>
+    <hyperlink ref="E91" r:id="rId90" display="roberto.soleti@dipc.org"/>
+    <hyperlink ref="E92" r:id="rId91" display="sorel@ific.uv.es"/>
+    <hyperlink ref="E93" r:id="rId92" display="josealfonso.soto@ific.uv.es"/>
+    <hyperlink ref="E94" r:id="rId93" display="steruel@ific.uv.es"/>
+    <hyperlink ref="E95" r:id="rId94" display="jtoledo@eln.upv.es"/>
+    <hyperlink ref="E96" r:id="rId95" display="claire.tonnele@dipc.org"/>
+    <hyperlink ref="E97" r:id="rId96" display="samuele.torelli@dipc.org"/>
+    <hyperlink ref="E98" r:id="rId97" display="jordi.torrent@udg.edu"/>
+    <hyperlink ref="F99" r:id="rId98" display="https://orcid.org/0000-0002-7621-5804"/>
+    <hyperlink ref="E100" r:id="rId99" display="alexandra.trettin@manchester.ac.uk"/>
+    <hyperlink ref="E101" r:id="rId100" display="pablo.garcia@dipc.org"/>
+    <hyperlink ref="E102" r:id="rId101" display="mukundam.vanga@uta.edu"/>
+    <hyperlink ref="E103" r:id="rId102" display="pablo.vazquez@dipc.org"/>
+    <hyperlink ref="F103" r:id="rId103" display="https://orcid.org/0009-0007-0098-8927"/>
+    <hyperlink ref="E104" r:id="rId104" display="joao.veloso@ua.pt"/>
+    <hyperlink ref="E105" r:id="rId105" display="Juan.Villamil@ific.uv.es"/>
+    <hyperlink ref="E106" r:id="rId106" display="john.waiton@postgrad.manchester.ac.uk"/>
+    <hyperlink ref="E107" r:id="rId107" display="alfonso.yubero@dipc.org"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>